<commit_message>
Actualizacion de casos de prueba
</commit_message>
<xml_diff>
--- a/alumnos/Fede_Bazan/TareaFecha13Y15/Demoblaze/Inicio de sesion/Caso de Prueba DemoBlaze Inicio Sesion.xlsx
+++ b/alumnos/Fede_Bazan/TareaFecha13Y15/Demoblaze/Inicio de sesion/Caso de Prueba DemoBlaze Inicio Sesion.xlsx
@@ -1,12 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Canavire\pythonCourse\QaAutomationCourseByPabloSoifer\RamaSeba\reporte-de-errores-informatorio\alumnos\Fede_Bazan\TareaFecha13Y15\Demoblaze\Inicio de sesion\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -263,183 +271,1195 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <font/>
+  <dxfs count="67">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4C7C3"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFB7E1CD"/>
           <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF4C7C3"/>
           <bgColor rgb="FFF4C7C3"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4DD0E1"/>
           <bgColor rgb="FF4DD0E1"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE0F7FA"/>
           <bgColor rgb="FFE0F7FA"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3F3F3"/>
+          <bgColor rgb="FFF3F3F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFBDBDBD"/>
           <bgColor rgb="FFBDBDBD"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF3F3F3"/>
-          <bgColor rgb="FFF3F3F3"/>
-        </patternFill>
-      </fill>
-      <border/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4DD0E1"/>
+          <bgColor rgb="FF4DD0E1"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="8">
-    <tableStyle count="3" pivot="0" name="Hoja 1-style">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="66"/>
+      <tableStyleElement type="firstRowStripe" dxfId="65"/>
+      <tableStyleElement type="secondRowStripe" dxfId="64"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 2">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 2" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="63"/>
+      <tableStyleElement type="firstRowStripe" dxfId="62"/>
+      <tableStyleElement type="secondRowStripe" dxfId="61"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 3">
-      <tableStyleElement dxfId="6" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="7" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 3" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="60"/>
+      <tableStyleElement type="firstRowStripe" dxfId="59"/>
+      <tableStyleElement type="secondRowStripe" dxfId="58"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 4">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 4" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="57"/>
+      <tableStyleElement type="firstRowStripe" dxfId="56"/>
+      <tableStyleElement type="secondRowStripe" dxfId="55"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 5">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 5" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="54"/>
+      <tableStyleElement type="firstRowStripe" dxfId="53"/>
+      <tableStyleElement type="secondRowStripe" dxfId="52"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 6">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 6" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="51"/>
+      <tableStyleElement type="firstRowStripe" dxfId="50"/>
+      <tableStyleElement type="secondRowStripe" dxfId="49"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 7">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 7" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="48"/>
+      <tableStyleElement type="firstRowStripe" dxfId="47"/>
+      <tableStyleElement type="secondRowStripe" dxfId="46"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Hoja 1-style 8">
-      <tableStyleElement dxfId="3" type="headerRow"/>
-      <tableStyleElement dxfId="4" type="firstRowStripe"/>
-      <tableStyleElement dxfId="5" type="secondRowStripe"/>
+    <tableStyle name="Hoja 1-style 8" pivot="0" count="3">
+      <tableStyleElement type="headerRow" dxfId="45"/>
+      <tableStyleElement type="firstRowStripe" dxfId="44"/>
+      <tableStyleElement type="secondRowStripe" dxfId="43"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:B1" displayName="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="A1:B1" headerRowCount="0" headerRowDxfId="26" dataDxfId="35" totalsRowDxfId="25">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="28"/>
+    <tableColumn id="2" name="Column2" dataDxfId="27"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -449,12 +1469,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A16:B16" displayName="Table_2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_2" displayName="Table_2" ref="A16:B16" headerRowCount="0" headerRowDxfId="22" dataDxfId="34" totalsRowDxfId="21">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="24"/>
+    <tableColumn id="2" name="Column2" dataDxfId="23"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -464,11 +1484,11 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B27" displayName="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_3" displayName="Table_3" ref="B27" headerRowCount="0" headerRowDxfId="38" dataDxfId="36" totalsRowDxfId="37">
   <tableColumns count="1">
-    <tableColumn name="Column1" id="1"/>
+    <tableColumn id="1" name="Column1" dataDxfId="20"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 3" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 3" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -478,12 +1498,12 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A31:B31" displayName="Table_4" id="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table_4" displayName="Table_4" ref="A31:B31" headerRowCount="0" headerRowDxfId="17" dataDxfId="33" totalsRowDxfId="16">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="19"/>
+    <tableColumn id="2" name="Column2" dataDxfId="18"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 4" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 4" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -493,12 +1513,12 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A46:B46" displayName="Table_5" id="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table_5" displayName="Table_5" ref="A46:B46" headerRowCount="0" headerRowDxfId="13" dataDxfId="32" totalsRowDxfId="12">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="15"/>
+    <tableColumn id="2" name="Column2" dataDxfId="14"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 5" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 5" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -508,12 +1528,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A61:B61" displayName="Table_6" id="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table_6" displayName="Table_6" ref="A61:B61" headerRowCount="0" headerRowDxfId="9" dataDxfId="31" totalsRowDxfId="8">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="11"/>
+    <tableColumn id="2" name="Column2" dataDxfId="10"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 6" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 6" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -523,12 +1543,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A76:B76" displayName="Table_7" id="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table_7" displayName="Table_7" ref="A76:B76" headerRowCount="0" headerRowDxfId="5" dataDxfId="30" totalsRowDxfId="4">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="7"/>
+    <tableColumn id="2" name="Column2" dataDxfId="6"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 7" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 7" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -538,12 +1558,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A91:B91" displayName="Table_8" id="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table_8" displayName="Table_8" ref="A91:B91" headerRowCount="0" headerRowDxfId="1" dataDxfId="29" totalsRowDxfId="0">
   <tableColumns count="2">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
+    <tableColumn id="1" name="Column1" dataDxfId="3"/>
+    <tableColumn id="2" name="Column2" dataDxfId="2"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style 8" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style 8" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -553,7 +1573,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -743,778 +1763,782 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B103"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.75"/>
+    <col min="1" max="1" width="23.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="96.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:2" ht="73.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:2" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="s">
+    <row r="33" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="s">
+    <row r="34" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="s">
+    <row r="35" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="s">
+    <row r="37" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="s">
+    <row r="38" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="s">
+    <row r="39" spans="1:2" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="s">
+    <row r="40" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="s">
+    <row r="41" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="s">
+    <row r="42" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="s">
+    <row r="43" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="s">
+    <row r="47" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="s">
+    <row r="48" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="s">
+    <row r="49" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="s">
+    <row r="51" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="s">
+    <row r="52" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="s">
+    <row r="53" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="s">
+    <row r="54" spans="1:2" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="s">
+    <row r="55" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="s">
+    <row r="56" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="s">
+    <row r="57" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="s">
+    <row r="58" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="1" t="s">
+    <row r="61" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A61" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="s">
+    <row r="62" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="s">
+    <row r="63" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A63" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="s">
+    <row r="64" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="s">
+    <row r="65" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="s">
+    <row r="66" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="s">
+    <row r="67" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="s">
+    <row r="68" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A68" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="s">
+    <row r="69" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="8" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2" t="s">
+    <row r="70" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="2" t="s">
+    <row r="71" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="2" t="s">
+    <row r="72" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="2" t="s">
+    <row r="73" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="1" t="s">
+    <row r="76" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A76" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="2" t="s">
+    <row r="77" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="2" t="s">
+    <row r="78" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="2" t="s">
+    <row r="79" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="2" t="s">
+    <row r="80" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="2" t="s">
+    <row r="81" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A81" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="2" t="s">
+    <row r="82" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="2" t="s">
+    <row r="83" spans="1:2" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="2" t="s">
+    <row r="84" spans="1:2" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="2" t="s">
+    <row r="85" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A85" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="s">
+    <row r="86" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A86" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="2" t="s">
+    <row r="87" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A87" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="2" t="s">
+    <row r="88" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A88" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="1" t="s">
+    <row r="91" spans="1:2" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A91" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" s="5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="2" t="s">
+    <row r="92" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A92" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="B92" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="2" t="s">
+    <row r="93" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A93" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B93" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="2" t="s">
+    <row r="94" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A94" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="2" t="s">
+    <row r="95" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B95" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="2" t="s">
+    <row r="96" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A96" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="2" t="s">
+    <row r="97" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="2" t="s">
+    <row r="98" spans="1:2" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="2" t="s">
+    <row r="99" spans="1:2" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="2" t="s">
+    <row r="100" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A100" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="2" t="s">
+    <row r="101" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A101" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="2" t="s">
+    <row r="102" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A102" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="2" t="s">
+    <row r="103" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A103" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" s="7" t="s">
         <v>71</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B27 B42 B12">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="1">
+    <cfRule type="notContainsBlanks" dxfId="42" priority="1">
       <formula>LEN(TRIM(B27))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57">
-    <cfRule type="notContainsBlanks" dxfId="1" priority="2">
+    <cfRule type="notContainsBlanks" dxfId="41" priority="2">
       <formula>LEN(TRIM(B57))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="3">
+    <cfRule type="notContainsBlanks" dxfId="40" priority="3">
       <formula>LEN(TRIM(B72))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87 B102">
-    <cfRule type="notContainsBlanks" dxfId="1" priority="4">
+    <cfRule type="notContainsBlanks" dxfId="39" priority="4">
       <formula>LEN(TRIM(B87))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="8">
-    <tablePart r:id="rId10"/>
-    <tablePart r:id="rId11"/>
-    <tablePart r:id="rId12"/>
-    <tablePart r:id="rId13"/>
-    <tablePart r:id="rId14"/>
-    <tablePart r:id="rId15"/>
-    <tablePart r:id="rId16"/>
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>